<commit_message>
Add staff profile defaults
</commit_message>
<xml_diff>
--- a/data/clients_template.xlsx
+++ b/data/clients_template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Information" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcedureSpecificData" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InsuranceData" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RM_Profile" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff_Profile" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk_CIS_Template" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -830,53 +830,104 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>rm_name</t>
+          <t>staff_name</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Shown in history GeneratedBy if provided</t>
+          <t>Default staff/RM name printed on forms</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>staff_id</t>
+          <t>staff_ic</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Staff IC if required by form</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fimm_id</t>
+          <t>staff_id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Staff ID</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ippc_id</t>
+          <t>fimm_id</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FIMM ID if required</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>branches</t>
+          <t>ippc_id</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Comma-separated, e.g. KJG,SUJ,KEL</t>
+          <t>IPPC ID if required</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>staff_position</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Example: Relationship Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>staff_rm_codes</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Comma-separated options, e.g. RM001,RM002</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>staff_branches</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Comma-separated options, e.g. KJG,SUJ,KEL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve mapping and procedure workflows
</commit_message>
<xml_diff>
--- a/data/clients_template.xlsx
+++ b/data/clients_template.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basic Information" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Information" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcedureSpecificData" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InsuranceData" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff_Profile" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk_CIS_Template" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="default_clients" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="default_accounts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="default_investment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="default_insurance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="default_staff" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bulk_cis_template" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="history_log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,7 +45,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,7 +63,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,92 +431,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>cis</t>
+          <t>*cis</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>*name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ic_number</t>
+          <t>*client_name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>policy_number</t>
+          <t>*ic_number</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>*policy_number</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>address_line1</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>address_line2</t>
+          <t>*address_line1</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>*address_line2</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>*city</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>postcode</t>
+          <t>*state</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>*postcode</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>branch_code</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>dob</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>occupation</t>
         </is>
@@ -532,56 +541,61 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Sample Customer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>900101101234</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>POL001</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>0123456789</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>sample@example.com</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Address line 1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>Kuala Lumpur</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>WP</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>50000</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>KJG</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>01/01/1990</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
@@ -598,58 +612,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>cis</t>
+          <t>common_name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>risk_profile</t>
+          <t>account_type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>investment_objective</t>
+          <t>account_number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>source_of_funds</t>
+          <t>holder_1_name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>annual_income</t>
+          <t>holder_1_cis</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>net_worth</t>
+          <t>holder_1_ic</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>sophisticated_investor</t>
+          <t>holder_2_name</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>holder_2_cis</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>holder_2_ic</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>holder_3_name</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>holder_3_cis</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>holder_3_ic</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>relationship_mode</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sample UT Main</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UT000001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sample Customer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CIS001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>900101101234</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>RHB</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Example account row</t>
         </is>
       </c>
     </row>
@@ -664,18 +780,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,40 +804,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>common_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>account_number</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>fd_details</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>product_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>action_purpose</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>follow_up_note</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fund_name</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>payment_method</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>bank_account_no</t>
         </is>
@@ -740,12 +868,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -802,134 +930,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>field</t>
+          <t>staff_name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>staff_ic</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>remarks</t>
+          <t>staff_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fimm_id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ippc_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>staff_position</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>staff_rm_codes</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>staff_branches</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>staff_name</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Default staff/RM name printed on forms</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>staff_ic</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Staff IC if required by form</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>staff_id</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Staff ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>fimm_id</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FIMM ID if required</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ippc_id</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>IPPC ID if required</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>staff_position</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Example: Relationship Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>staff_rm_codes</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Comma-separated options, e.g. RM001,RM002</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>staff_branches</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Comma-separated options, e.g. KJG,SUJ,KEL</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -958,4 +1022,106 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GeneratedDateTime</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ClientName</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ProcedureCode</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ProcedureName</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>OutputFilePath</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FDDetails</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ProductType</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ActionPurpose</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>FollowUpNote</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ErrorMessage</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>GeneratedBy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>